<commit_message>
Sushi Restaurant Business Plan Kit EN · F2 (WIP): los 4 entregables EN en dl/ (G1-G9 TODO VERDE, autotests 20/20 y 8/8, calculadora 585 VERDE, barrido 1,718 piezas 0 fallos, censo --letter 0, no latinos 0, LIT255 verde)
Via: Claude Code
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/sushi-restaurant-business-plan/sushi-restaurant-financial-projections.xlsx
+++ b/astro-site/public/dl/sushi-restaurant-business-plan/sushi-restaurant-financial-projections.xlsx
@@ -826,7 +826,7 @@
         <v>35.1</v>
       </c>
       <c r="C9" t="str">
-        <f>IFERROR("Average check excl. sales tax plus the weighted sales tax of your sales lines ("&amp;TEXT(SUMPRODUCT('3-Year P&amp;L'!$E$10:$E$11,'3-Year P&amp;L'!$G$10:$G$11)*100,"0")&amp;"%), rounded. In the US, menu prices usually exclude sales tax and it is added at the register; the beverage share in column H of the beverage line of the P&amp;L only moves this average if your state taxes alcohol at another rate. In the UK, "&amp;"menu prices include VAT.","")</f>
+        <f>IFERROR("Average check excl. sales tax plus the weighted sales tax of your sales lines ("&amp;TEXT(SUMPRODUCT('3-Year P&amp;L'!$E$10:$E$11,'3-Year P&amp;L'!$G$10:$G$11)*100,"0")&amp;"%), rounded. In the US, menu prices usually exclude sales tax and it is added at the register; the beverage share in column H of the beverage line of the P&amp;L only moves this average if your state taxes alcohol at another rate. "&amp;"In the UK, menu prices include VAT.","")</f>
         <v>Average check excl. sales tax plus the weighted sales tax of your sales lines (8%), rounded. In the US, menu prices usually exclude sales tax and it is added at the register; the beverage share in column H of the beverage line of the P&amp;L only moves this average if your state taxes alcohol at another rate. In the UK, menu prices include VAT.</v>
       </c>
     </row>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="B38" s="29" t="inlineStr">
         <is>
-          <t>Theoretical cost of each nigiri, roll and platter by channel</t>
+          <t>Salmon nigiri about 23%, California roll about 12%, spicy tuna roll about 39%; whole menu about 24%</t>
         </is>
       </c>
       <c r="C38" s="29" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="D38" s="48" t="inlineStr">
         <is>
-          <t>The plan's 32% is the real usage of the whole menu, waste included, so it comes out higher than the cost per piece</t>
+          <t>The plan's 32% is the real usage of the whole menu, with case shrink, trim, rice thrown out and staff meals: it comes out higher than the theoretical cost per piece</t>
         </is>
       </c>
       <c r="E38" s="29" t="n"/>

</xml_diff>